<commit_message>
Add footer block, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files: 20
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-adventures.report.xlsx
+++ b/tools/importer/reports/import-adventures.report.xlsx
@@ -154,7 +154,7 @@
     <t>adventures</t>
   </si>
   <si>
-    <t>2026-09-24T16:00:33.965Z</t>
+    <t>2026-09-24T17:43:21.610Z</t>
   </si>
   <si>
     <t>Bali Surf Camp</t>
@@ -169,7 +169,7 @@
     <t>us/en/adventures/beervana-portland</t>
   </si>
   <si>
-    <t>2026-09-24T16:00:39.610Z</t>
+    <t>2026-09-24T17:43:26.368Z</t>
   </si>
   <si>
     <t>Beervana in Portland</t>
@@ -184,7 +184,7 @@
     <t>us/en/adventures/climbing-new-zealand</t>
   </si>
   <si>
-    <t>2026-09-24T16:00:44.376Z</t>
+    <t>2026-09-24T17:43:33.082Z</t>
   </si>
   <si>
     <t>Climbing New Zealand</t>
@@ -199,7 +199,7 @@
     <t>us/en/adventures/colorado-rock-climbing</t>
   </si>
   <si>
-    <t>2026-09-24T16:00:49.658Z</t>
+    <t>2026-09-24T17:43:39.159Z</t>
   </si>
   <si>
     <t>Colorado Rock Climbing</t>
@@ -214,7 +214,7 @@
     <t>us/en/adventures/cycling-southern-utah</t>
   </si>
   <si>
-    <t>2026-09-24T16:00:53.684Z</t>
+    <t>2026-09-24T17:43:43.820Z</t>
   </si>
   <si>
     <t>Cycling Southern Utah</t>
@@ -229,7 +229,7 @@
     <t>us/en/adventures/cycling-tuscany</t>
   </si>
   <si>
-    <t>2026-09-24T16:00:58.206Z</t>
+    <t>2026-09-24T17:43:49.271Z</t>
   </si>
   <si>
     <t>Cycling Tuscany</t>
@@ -244,7 +244,7 @@
     <t>us/en/adventures/downhill-skiing-wyoming</t>
   </si>
   <si>
-    <t>2026-09-24T16:01:04.334Z</t>
+    <t>2026-09-24T17:43:54.492Z</t>
   </si>
   <si>
     <t>Downhill Skiing Wyoming</t>
@@ -259,7 +259,7 @@
     <t>us/en/adventures/gastronomic-marais-tour</t>
   </si>
   <si>
-    <t>2026-09-24T16:01:10.599Z</t>
+    <t>2026-09-24T17:43:59.547Z</t>
   </si>
   <si>
     <t>Gastronomic Marais Tour</t>
@@ -274,7 +274,7 @@
     <t>us/en/adventures/napa-wine-tasting</t>
   </si>
   <si>
-    <t>2026-09-24T16:01:15.203Z</t>
+    <t>2026-09-24T17:44:03.788Z</t>
   </si>
   <si>
     <t>Napa Wine Tasting</t>
@@ -289,7 +289,7 @@
     <t>us/en/adventures/riverside-camping-australia</t>
   </si>
   <si>
-    <t>2026-09-24T16:01:19.277Z</t>
+    <t>2026-09-24T17:44:09.511Z</t>
   </si>
   <si>
     <t>Riverside Camping</t>
@@ -304,7 +304,7 @@
     <t>us/en/adventures/ski-touring-mont-blanc</t>
   </si>
   <si>
-    <t>2026-09-24T16:01:24.612Z</t>
+    <t>2026-09-24T17:44:14.698Z</t>
   </si>
   <si>
     <t>Ski Touring Mont Blanc</t>
@@ -319,7 +319,7 @@
     <t>us/en/adventures/surf-camp-costa-rica</t>
   </si>
   <si>
-    <t>2026-09-24T16:01:28.561Z</t>
+    <t>2026-09-24T17:44:18.859Z</t>
   </si>
   <si>
     <t>Surf Camp in Costa Rica</t>
@@ -334,7 +334,7 @@
     <t>us/en/adventures/tahoe-skiing</t>
   </si>
   <si>
-    <t>2026-09-24T16:01:32.876Z</t>
+    <t>2026-09-24T17:44:24.577Z</t>
   </si>
   <si>
     <t>Tahoe Skiing</t>
@@ -349,7 +349,7 @@
     <t>us/en/adventures/west-coast-cycling</t>
   </si>
   <si>
-    <t>2026-09-24T16:01:38.035Z</t>
+    <t>2026-09-24T17:44:30.024Z</t>
   </si>
   <si>
     <t>West Coast Cycling</t>
@@ -364,7 +364,7 @@
     <t>us/en/adventures/whistler-mountain-biking</t>
   </si>
   <si>
-    <t>2026-09-24T16:01:44.722Z</t>
+    <t>2026-09-24T17:44:34.938Z</t>
   </si>
   <si>
     <t>Whistler Mountain Biking</t>
@@ -379,7 +379,7 @@
     <t>us/en/adventures/yosemite-backpacking</t>
   </si>
   <si>
-    <t>2026-09-24T16:01:49.580Z</t>
+    <t>2026-09-24T17:44:40.162Z</t>
   </si>
   <si>
     <t>Yosemite Backpacking</t>

</xml_diff>